<commit_message>
update 2023 and 2024 to v2.5; Minor Updates in GNFR C
</commit_message>
<xml_diff>
--- a/output/2023/sector_totals_2023.xlsx
+++ b/output/2023/sector_totals_2023.xlsx
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1733.439382439184</v>
+        <v>1455.722107292333</v>
       </c>
       <c r="C3" t="n">
-        <v>114.9055299929168</v>
+        <v>103.9850228864146</v>
       </c>
       <c r="D3" t="n">
-        <v>691.4897039261906</v>
+        <v>584.1940258671902</v>
       </c>
       <c r="E3" t="n">
-        <v>2141.270884832333</v>
+        <v>1908.467732705251</v>
       </c>
       <c r="F3" t="n">
-        <v>183.0528173406445</v>
+        <v>157.737357387463</v>
       </c>
       <c r="G3" t="n">
-        <v>85.75107534256469</v>
+        <v>78.00271512360187</v>
       </c>
     </row>
     <row r="4">
@@ -817,22 +817,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6068.242994830194</v>
+        <v>5790.525719683343</v>
       </c>
       <c r="C16" t="n">
-        <v>973.5278710254981</v>
+        <v>962.6073639189958</v>
       </c>
       <c r="D16" t="n">
-        <v>4257.826985529312</v>
+        <v>4150.531307470312</v>
       </c>
       <c r="E16" t="n">
-        <v>8567.062439069236</v>
+        <v>8334.259286942153</v>
       </c>
       <c r="F16" t="n">
-        <v>1673.926704693204</v>
+        <v>1648.611244740022</v>
       </c>
       <c r="G16" t="n">
-        <v>113.1958263481406</v>
+        <v>105.4474661291777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>